<commit_message>
GBDS JUNE 2026 | berlyn@gbds
</commit_message>
<xml_diff>
--- a/GBDS JUNE FILES 2026/MONTHLY DIS TO DO/DIS MONTHLY REPORTS.xlsx
+++ b/GBDS JUNE FILES 2026/MONTHLY DIS TO DO/DIS MONTHLY REPORTS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS 2024\GBDS AUG FILES 2024\DIS Aug\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS JUNE FILES 2026\MONTHLY DIS TO DO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D31CF38F-F699-40EC-83BA-F27DF502DE4D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F1201C9-3C67-48F8-B82C-8C5683943B1D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F0893456-6701-4EDC-85B3-E0F891996231}"/>
   </bookViews>
@@ -156,40 +156,40 @@
     <t>SIR NEIL SMS</t>
   </si>
   <si>
-    <t>1-8</t>
-  </si>
-  <si>
-    <t>9-16</t>
-  </si>
-  <si>
-    <t>17-23</t>
-  </si>
-  <si>
-    <t>24-30</t>
-  </si>
-  <si>
-    <t>MAY 2026</t>
-  </si>
-  <si>
-    <t>ANALYTICS ALL PRODUCTS MAY</t>
-  </si>
-  <si>
-    <t>ANALYTICS ALL PRODUCTS JAN-MAY</t>
-  </si>
-  <si>
-    <t>ANALYTICS BEER MAY</t>
-  </si>
-  <si>
-    <t>ANALYTICS BEER JAN TO MAY</t>
-  </si>
-  <si>
-    <t>ANALYTICS NAB MAY</t>
-  </si>
-  <si>
-    <t>ANALYTICS NAB JAN TO MAY</t>
-  </si>
-  <si>
     <t>a</t>
+  </si>
+  <si>
+    <t>JUNE 2026</t>
+  </si>
+  <si>
+    <t>ANALYTICS ALL PRODUCTS JUNE</t>
+  </si>
+  <si>
+    <t>ANALYTICS ALL PRODUCTS JAN-JUNE</t>
+  </si>
+  <si>
+    <t>ANALYTICS BEER JUNE</t>
+  </si>
+  <si>
+    <t>ANALYTICS BEER JAN TO JUNE</t>
+  </si>
+  <si>
+    <t>ANALYTICS NAB JUNE</t>
+  </si>
+  <si>
+    <t>ANALYTICS NAB JAN TO JUNE</t>
+  </si>
+  <si>
+    <t>1-7</t>
+  </si>
+  <si>
+    <t>8-14</t>
+  </si>
+  <si>
+    <t>15-21</t>
+  </si>
+  <si>
+    <t>22-30</t>
   </si>
 </sst>
 </file>
@@ -586,7 +586,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -604,10 +604,10 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s">
         <v>39</v>
@@ -619,10 +619,10 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E7" t="s">
         <v>39</v>
@@ -634,10 +634,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E8" t="s">
         <v>39</v>
@@ -649,10 +649,10 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E9" t="s">
         <v>39</v>
@@ -664,10 +664,10 @@
         <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E10" t="s">
         <v>39</v>
@@ -679,10 +679,10 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E11" t="s">
         <v>39</v>
@@ -706,7 +706,7 @@
         <v>2</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E13" t="s">
         <v>39</v>
@@ -721,7 +721,7 @@
         <v>3</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E14" t="s">
         <v>39</v>
@@ -741,10 +741,10 @@
         <v>16</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E16" t="s">
         <v>39</v>
@@ -759,10 +759,10 @@
         <v>17</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E17" t="s">
         <v>39</v>
@@ -777,10 +777,10 @@
         <v>18</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E18" t="s">
         <v>39</v>
@@ -795,10 +795,10 @@
         <v>19</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E19" t="s">
         <v>39</v>
@@ -821,7 +821,7 @@
         <v>7</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
@@ -839,7 +839,7 @@
         <v>5</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
@@ -857,7 +857,7 @@
         <v>6</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
@@ -878,7 +878,7 @@
         <v>8</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
@@ -896,7 +896,7 @@
         <v>9</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
@@ -914,7 +914,7 @@
         <v>10</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:18" ht="16.5" x14ac:dyDescent="0.25">
@@ -932,7 +932,7 @@
         <v>11</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>33</v>
@@ -970,7 +970,7 @@
         <v>22</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38" spans="1:18" ht="16.5" x14ac:dyDescent="0.25">
@@ -982,7 +982,7 @@
         <v>23</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="39" spans="1:18" ht="16.5" x14ac:dyDescent="0.25">
@@ -994,7 +994,7 @@
         <v>24</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
@@ -1008,7 +1008,7 @@
         <v>13</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E41" t="s">
         <v>26</v>
@@ -1031,7 +1031,7 @@
         <v>15</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E43" t="s">
         <v>29</v>

</xml_diff>